<commit_message>
Report: add Scenario column to Known Prod Defects; spillover list cleanup
- report.html: add Scenario as first column in the Known Production Defects table
- spillover.html: remove Type column from list view, fix empty-state colspan
- config: switch downloads_folder to laptop path
- output: updated retail_report_log.xlsx
- add planning prompt MDs for retail steps 1-3, retail report step 1, spillover fix

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/retail_report_log.xlsx
+++ b/output/retail_report_log.xlsx
@@ -539,35 +539,35 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D4" t="n">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="E4" t="n">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>